<commit_message>
Fix save-sheet endpoint preserving styles and layout
</commit_message>
<xml_diff>
--- a/backend/Rwanda/fuel-financial-inputs.xlsx
+++ b/backend/Rwanda/fuel-financial-inputs.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet name="LPG" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Electricity" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Carbon Credits" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
@@ -930,4 +931,282 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Inputs</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D1" s="8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E1" s="8" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F1" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G1" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="H1" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="I1" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="J1" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="K1" s="8" t="n">
+        <v>2031</v>
+      </c>
+      <c r="L1" s="8" t="n">
+        <v>2032</v>
+      </c>
+      <c r="M1" s="8" t="n">
+        <v>2033</v>
+      </c>
+      <c r="N1" s="8" t="n">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>CO2 certificate (%) - from the total CO2 avoided</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Liquidity</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Price per TON</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>$ / ton</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Number of years that you could sell those carbon credits</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Prevent false cache hits for same-label cross-file sources
- Only use cache when source label matches target AND files are the same

- Fixes issue where external inputs (e.g. fuel-financial-inputs.xlsx) were incorrectly served from cache
</commit_message>
<xml_diff>
--- a/backend/Rwanda/fuel-financial-inputs.xlsx
+++ b/backend/Rwanda/fuel-financial-inputs.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LPG" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Electricity" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Electricity" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LPG" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1" iterate="1"/>
 </workbook>
 </file>
 
@@ -102,24 +102,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -516,23 +501,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Hoja2">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="31.6640625" customWidth="1" min="1" max="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" ht="16.05" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
@@ -574,147 +556,147 @@
         <v>2034</v>
       </c>
     </row>
-    <row r="2" ht="16.05" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Expected non-technical losses</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="I2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="J2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="K2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N2" s="6" t="n">
+      <c r="C2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="M2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="N2" s="1" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="16.05" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Trade receivables - Days of revenues</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>days</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="G3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="I3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="J3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="K3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="L3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="M3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="N3" s="6" t="n">
+      <c r="C3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="M3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="N3" s="1" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="4" ht="16.05" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Trade payables - Days of OPEX costs</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>days</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="I4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="K4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="L4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="M4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="N4" s="6" t="n">
+      <c r="C4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="M4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="N4" s="1" t="n">
         <v>30</v>
       </c>
     </row>
@@ -730,200 +712,200 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="34.77734375" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.6" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="C1" s="8" t="n">
+      <c r="C1" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="D1" s="8" t="n">
+      <c r="D1" s="3" t="n">
         <v>2024</v>
       </c>
-      <c r="E1" s="8" t="n">
+      <c r="E1" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="F1" s="8" t="n">
+      <c r="F1" s="3" t="n">
         <v>2026</v>
       </c>
-      <c r="G1" s="8" t="n">
+      <c r="G1" s="3" t="n">
         <v>2027</v>
       </c>
-      <c r="H1" s="8" t="n">
+      <c r="H1" s="3" t="n">
         <v>2028</v>
       </c>
-      <c r="I1" s="8" t="n">
+      <c r="I1" s="3" t="n">
         <v>2029</v>
       </c>
-      <c r="J1" s="8" t="n">
+      <c r="J1" s="3" t="n">
         <v>2030</v>
       </c>
-      <c r="K1" s="8" t="n">
+      <c r="K1" s="3" t="n">
         <v>2031</v>
       </c>
-      <c r="L1" s="8" t="n">
+      <c r="L1" s="3" t="n">
         <v>2032</v>
       </c>
-      <c r="M1" s="8" t="n">
+      <c r="M1" s="3" t="n">
         <v>2033</v>
       </c>
-      <c r="N1" s="8" t="n">
+      <c r="N1" s="3" t="n">
         <v>2034</v>
       </c>
     </row>
-    <row r="2" ht="15.6" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Expected non-technical losses</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N2" s="4" t="n">
+      <c r="C2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="M2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="N2" s="1" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="15.6" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Trade receivables - Days of revenues</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>days</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="K3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="L3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="M3" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="N3" s="4" t="n">
+      <c r="C3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="M3" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="N3" s="1" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="4" ht="15.6" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Trade payables - Days of OPEX costs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>days</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="N4" s="4" t="n">
+      <c r="C4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="M4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="N4" s="1" t="n">
         <v>30</v>
       </c>
     </row>

</xml_diff>